<commit_message>
Update report card template to show average, general average, and passed or fail indications if 4th grading grades are not empty
</commit_message>
<xml_diff>
--- a/public/files/report_card_templates/Grade1-3.xlsx
+++ b/public/files/report_card_templates/Grade1-3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BTCSI\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\schoolsys\public\files\report_card_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74599A78-F372-4030-B3E4-E60E2D98FC9B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29F6716-E47B-423D-89D6-363645B85D05}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="71">
   <si>
     <t>PROGRESS REPORT</t>
   </si>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>FILIPINO</t>
-  </si>
-  <si>
-    <t>Passed</t>
   </si>
   <si>
     <t>ENGLISH</t>
@@ -430,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -551,15 +548,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -572,6 +569,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -802,7 +803,9 @@
   <dimension ref="A1:AN1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="40" width="1.5703125" customWidth="1"/>
+    <col min="1" max="27" width="1.5703125" customWidth="1"/>
+    <col min="28" max="28" width="2.140625" customWidth="1"/>
+    <col min="29" max="40" width="1.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:40" ht="12.75" customHeight="1">
@@ -1077,17 +1080,18 @@
       <c r="AA7" s="17"/>
       <c r="AB7" s="17"/>
       <c r="AC7" s="15"/>
-      <c r="AD7" s="41">
-        <f t="shared" ref="AD7:AD18" si="0">SUM(N7:AC7)/4</f>
-        <v>0</v>
+      <c r="AD7" s="41" t="str">
+        <f>IF(COUNT(N7:AC7)=4,SUM(N7:AC7)/4,"")</f>
+        <v/>
       </c>
       <c r="AE7" s="17"/>
       <c r="AF7" s="17"/>
       <c r="AG7" s="17"/>
       <c r="AH7" s="17"/>
       <c r="AI7" s="15"/>
-      <c r="AJ7" s="35" t="s">
-        <v>16</v>
+      <c r="AJ7" s="35" t="str">
+        <f>IF(AD7&lt;&gt;"",IF(AD7&gt;=75,"Passed","Failed"),"")</f>
+        <v/>
       </c>
       <c r="AK7" s="17"/>
       <c r="AL7" s="17"/>
@@ -1096,7 +1100,7 @@
     </row>
     <row r="8" spans="1:40" ht="12.75" customHeight="1">
       <c r="A8" s="40" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -1126,17 +1130,18 @@
       <c r="AA8" s="17"/>
       <c r="AB8" s="17"/>
       <c r="AC8" s="15"/>
-      <c r="AD8" s="41">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="AD8" s="41" t="str">
+        <f t="shared" ref="AD8:AD20" si="0">IF(COUNT(N8:AC8)=4,SUM(N8:AC8)/4,"")</f>
+        <v/>
       </c>
       <c r="AE8" s="17"/>
       <c r="AF8" s="17"/>
       <c r="AG8" s="17"/>
       <c r="AH8" s="17"/>
       <c r="AI8" s="15"/>
-      <c r="AJ8" s="35" t="s">
-        <v>16</v>
+      <c r="AJ8" s="35" t="str">
+        <f t="shared" ref="AJ8:AJ20" si="1">IF(AD8&lt;&gt;"",IF(AD8&gt;=75,"Passed","Failed"),"")</f>
+        <v/>
       </c>
       <c r="AK8" s="17"/>
       <c r="AL8" s="17"/>
@@ -1145,7 +1150,7 @@
     </row>
     <row r="9" spans="1:40" ht="12.75" customHeight="1">
       <c r="A9" s="40" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1175,17 +1180,18 @@
       <c r="AA9" s="17"/>
       <c r="AB9" s="17"/>
       <c r="AC9" s="15"/>
-      <c r="AD9" s="41">
+      <c r="AD9" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE9" s="17"/>
       <c r="AF9" s="17"/>
       <c r="AG9" s="17"/>
       <c r="AH9" s="17"/>
       <c r="AI9" s="15"/>
-      <c r="AJ9" s="35" t="s">
-        <v>16</v>
+      <c r="AJ9" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK9" s="17"/>
       <c r="AL9" s="17"/>
@@ -1194,7 +1200,7 @@
     </row>
     <row r="10" spans="1:40" ht="12.75" customHeight="1">
       <c r="A10" s="40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -1224,17 +1230,18 @@
       <c r="AA10" s="17"/>
       <c r="AB10" s="17"/>
       <c r="AC10" s="15"/>
-      <c r="AD10" s="41">
+      <c r="AD10" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE10" s="17"/>
       <c r="AF10" s="17"/>
       <c r="AG10" s="17"/>
       <c r="AH10" s="17"/>
       <c r="AI10" s="15"/>
-      <c r="AJ10" s="35" t="s">
-        <v>16</v>
+      <c r="AJ10" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK10" s="17"/>
       <c r="AL10" s="17"/>
@@ -1243,7 +1250,7 @@
     </row>
     <row r="11" spans="1:40" ht="12.75" customHeight="1">
       <c r="A11" s="40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1273,17 +1280,18 @@
       <c r="AA11" s="17"/>
       <c r="AB11" s="17"/>
       <c r="AC11" s="15"/>
-      <c r="AD11" s="41">
+      <c r="AD11" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE11" s="17"/>
       <c r="AF11" s="17"/>
       <c r="AG11" s="17"/>
       <c r="AH11" s="17"/>
       <c r="AI11" s="15"/>
-      <c r="AJ11" s="35" t="s">
-        <v>16</v>
+      <c r="AJ11" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK11" s="17"/>
       <c r="AL11" s="17"/>
@@ -1292,7 +1300,7 @@
     </row>
     <row r="12" spans="1:40" ht="12.75" customHeight="1">
       <c r="A12" s="40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -1322,17 +1330,18 @@
       <c r="AA12" s="17"/>
       <c r="AB12" s="17"/>
       <c r="AC12" s="15"/>
-      <c r="AD12" s="41">
+      <c r="AD12" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE12" s="17"/>
       <c r="AF12" s="17"/>
       <c r="AG12" s="17"/>
       <c r="AH12" s="17"/>
       <c r="AI12" s="15"/>
-      <c r="AJ12" s="35" t="s">
-        <v>16</v>
+      <c r="AJ12" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK12" s="17"/>
       <c r="AL12" s="17"/>
@@ -1341,8 +1350,8 @@
     </row>
     <row r="13" spans="1:40" ht="12.75" customHeight="1">
       <c r="A13" s="2"/>
-      <c r="B13" s="55" t="s">
-        <v>22</v>
+      <c r="B13" s="57" t="s">
+        <v>21</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
@@ -1355,7 +1364,7 @@
       <c r="K13" s="17"/>
       <c r="L13" s="17"/>
       <c r="M13" s="15"/>
-      <c r="N13" s="56"/>
+      <c r="N13" s="58"/>
       <c r="O13" s="17"/>
       <c r="P13" s="17"/>
       <c r="Q13" s="15"/>
@@ -1371,17 +1380,18 @@
       <c r="AA13" s="17"/>
       <c r="AB13" s="17"/>
       <c r="AC13" s="15"/>
-      <c r="AD13" s="41">
+      <c r="AD13" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE13" s="17"/>
       <c r="AF13" s="17"/>
       <c r="AG13" s="17"/>
       <c r="AH13" s="17"/>
       <c r="AI13" s="15"/>
-      <c r="AJ13" s="35" t="s">
-        <v>16</v>
+      <c r="AJ13" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK13" s="17"/>
       <c r="AL13" s="17"/>
@@ -1390,8 +1400,8 @@
     </row>
     <row r="14" spans="1:40" ht="12.75" customHeight="1">
       <c r="A14" s="2"/>
-      <c r="B14" s="55" t="s">
-        <v>23</v>
+      <c r="B14" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
@@ -1404,7 +1414,7 @@
       <c r="K14" s="17"/>
       <c r="L14" s="17"/>
       <c r="M14" s="15"/>
-      <c r="N14" s="56"/>
+      <c r="N14" s="58"/>
       <c r="O14" s="17"/>
       <c r="P14" s="17"/>
       <c r="Q14" s="15"/>
@@ -1420,17 +1430,18 @@
       <c r="AA14" s="17"/>
       <c r="AB14" s="17"/>
       <c r="AC14" s="15"/>
-      <c r="AD14" s="41">
+      <c r="AD14" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE14" s="17"/>
       <c r="AF14" s="17"/>
       <c r="AG14" s="17"/>
       <c r="AH14" s="17"/>
       <c r="AI14" s="15"/>
-      <c r="AJ14" s="35" t="s">
-        <v>16</v>
+      <c r="AJ14" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK14" s="17"/>
       <c r="AL14" s="17"/>
@@ -1439,8 +1450,8 @@
     </row>
     <row r="15" spans="1:40" ht="12.75" customHeight="1">
       <c r="A15" s="2"/>
-      <c r="B15" s="55" t="s">
-        <v>24</v>
+      <c r="B15" s="57" t="s">
+        <v>23</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
@@ -1453,7 +1464,7 @@
       <c r="K15" s="17"/>
       <c r="L15" s="17"/>
       <c r="M15" s="15"/>
-      <c r="N15" s="56"/>
+      <c r="N15" s="58"/>
       <c r="O15" s="17"/>
       <c r="P15" s="17"/>
       <c r="Q15" s="15"/>
@@ -1469,17 +1480,18 @@
       <c r="AA15" s="17"/>
       <c r="AB15" s="17"/>
       <c r="AC15" s="15"/>
-      <c r="AD15" s="41">
+      <c r="AD15" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE15" s="17"/>
       <c r="AF15" s="17"/>
       <c r="AG15" s="17"/>
       <c r="AH15" s="17"/>
       <c r="AI15" s="15"/>
-      <c r="AJ15" s="35" t="s">
-        <v>16</v>
+      <c r="AJ15" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK15" s="17"/>
       <c r="AL15" s="17"/>
@@ -1488,8 +1500,8 @@
     </row>
     <row r="16" spans="1:40" ht="12.75" customHeight="1">
       <c r="A16" s="2"/>
-      <c r="B16" s="55" t="s">
-        <v>25</v>
+      <c r="B16" s="57" t="s">
+        <v>24</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
@@ -1502,7 +1514,7 @@
       <c r="K16" s="17"/>
       <c r="L16" s="17"/>
       <c r="M16" s="15"/>
-      <c r="N16" s="56"/>
+      <c r="N16" s="58"/>
       <c r="O16" s="17"/>
       <c r="P16" s="17"/>
       <c r="Q16" s="15"/>
@@ -1518,17 +1530,18 @@
       <c r="AA16" s="17"/>
       <c r="AB16" s="17"/>
       <c r="AC16" s="15"/>
-      <c r="AD16" s="41">
+      <c r="AD16" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE16" s="17"/>
       <c r="AF16" s="17"/>
       <c r="AG16" s="17"/>
       <c r="AH16" s="17"/>
       <c r="AI16" s="15"/>
-      <c r="AJ16" s="35" t="s">
-        <v>16</v>
+      <c r="AJ16" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK16" s="17"/>
       <c r="AL16" s="17"/>
@@ -1537,7 +1550,7 @@
     </row>
     <row r="17" spans="1:40" ht="12.75" customHeight="1">
       <c r="A17" s="40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -1567,17 +1580,18 @@
       <c r="AA17" s="17"/>
       <c r="AB17" s="17"/>
       <c r="AC17" s="15"/>
-      <c r="AD17" s="41">
+      <c r="AD17" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE17" s="17"/>
       <c r="AF17" s="17"/>
       <c r="AG17" s="17"/>
       <c r="AH17" s="17"/>
       <c r="AI17" s="15"/>
-      <c r="AJ17" s="35" t="s">
-        <v>16</v>
+      <c r="AJ17" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK17" s="17"/>
       <c r="AL17" s="17"/>
@@ -1586,7 +1600,7 @@
     </row>
     <row r="18" spans="1:40" ht="12.75" customHeight="1">
       <c r="A18" s="40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -1616,17 +1630,18 @@
       <c r="AA18" s="17"/>
       <c r="AB18" s="17"/>
       <c r="AC18" s="15"/>
-      <c r="AD18" s="41">
+      <c r="AD18" s="41" t="str">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="AE18" s="17"/>
       <c r="AF18" s="17"/>
       <c r="AG18" s="17"/>
       <c r="AH18" s="17"/>
       <c r="AI18" s="15"/>
-      <c r="AJ18" s="35" t="s">
-        <v>16</v>
+      <c r="AJ18" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK18" s="17"/>
       <c r="AL18" s="17"/>
@@ -1635,7 +1650,7 @@
     </row>
     <row r="19" spans="1:40" ht="12.75" customHeight="1">
       <c r="A19" s="40" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -1665,13 +1680,19 @@
       <c r="AA19" s="17"/>
       <c r="AB19" s="17"/>
       <c r="AC19" s="15"/>
-      <c r="AD19" s="41"/>
+      <c r="AD19" s="41" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="AE19" s="17"/>
       <c r="AF19" s="17"/>
       <c r="AG19" s="17"/>
       <c r="AH19" s="17"/>
       <c r="AI19" s="15"/>
-      <c r="AJ19" s="35"/>
+      <c r="AJ19" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
       <c r="AK19" s="17"/>
       <c r="AL19" s="17"/>
       <c r="AM19" s="17"/>
@@ -1679,7 +1700,7 @@
     </row>
     <row r="20" spans="1:40" ht="12.75" customHeight="1">
       <c r="A20" s="40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -1709,17 +1730,18 @@
       <c r="AA20" s="17"/>
       <c r="AB20" s="17"/>
       <c r="AC20" s="15"/>
-      <c r="AD20" s="41">
-        <f>SUM(N20:AC20)/4</f>
-        <v>0</v>
+      <c r="AD20" s="41" t="str">
+        <f t="shared" si="0"/>
+        <v/>
       </c>
       <c r="AE20" s="17"/>
       <c r="AF20" s="17"/>
       <c r="AG20" s="17"/>
       <c r="AH20" s="17"/>
       <c r="AI20" s="15"/>
-      <c r="AJ20" s="35" t="s">
-        <v>16</v>
+      <c r="AJ20" s="35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
       </c>
       <c r="AK20" s="17"/>
       <c r="AL20" s="17"/>
@@ -1729,8 +1751,8 @@
     <row r="21" spans="1:40" ht="12.75" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" s="3"/>
-      <c r="C21" s="57" t="s">
-        <v>30</v>
+      <c r="C21" s="59" t="s">
+        <v>29</v>
       </c>
       <c r="D21" s="17"/>
       <c r="E21" s="17"/>
@@ -1742,43 +1764,41 @@
       <c r="K21" s="17"/>
       <c r="L21" s="17"/>
       <c r="M21" s="15"/>
-      <c r="N21" s="19">
-        <f>(+N7+N8+N9+N10+N11+N12+N17+N18)/8</f>
-        <v>0</v>
+      <c r="N21" s="19" t="str">
+        <f>IF($AD22&lt;&gt;"", SUM(N7:Q12,N17:Q18)/8,"")</f>
+        <v/>
       </c>
       <c r="O21" s="17"/>
       <c r="P21" s="17"/>
       <c r="Q21" s="15"/>
-      <c r="R21" s="19">
-        <f>(+R7+R8+R9+R10+R11+R12+R17+R18)/8</f>
-        <v>0</v>
+      <c r="R21" s="19" t="str">
+        <f t="shared" ref="R21" si="2">IF($AD22&lt;&gt;"", SUM(R7:U12,R17:U18)/8,"")</f>
+        <v/>
       </c>
       <c r="S21" s="17"/>
       <c r="T21" s="17"/>
       <c r="U21" s="15"/>
-      <c r="V21" s="19">
-        <f>(+V7+V8+V9+V10+V11+V12+V17+V18)/8</f>
-        <v>0</v>
+      <c r="V21" s="19" t="str">
+        <f t="shared" ref="V21" si="3">IF($AD22&lt;&gt;"", SUM(V7:Y12,V17:Y18)/8,"")</f>
+        <v/>
       </c>
       <c r="W21" s="17"/>
       <c r="X21" s="17"/>
       <c r="Y21" s="15"/>
-      <c r="Z21" s="19">
-        <f>(+Z7+Z8+Z9+Z10+Z11+Z12+Z17+Z18)/8</f>
-        <v>0</v>
+      <c r="Z21" s="19" t="str">
+        <f t="shared" ref="Z21" si="4">IF($AD22&lt;&gt;"", SUM(Z7:AC12,Z17:AC18)/8,"")</f>
+        <v/>
       </c>
       <c r="AA21" s="17"/>
       <c r="AB21" s="17"/>
       <c r="AC21" s="15"/>
-      <c r="AD21" s="58"/>
+      <c r="AD21" s="60"/>
       <c r="AE21" s="17"/>
       <c r="AF21" s="17"/>
       <c r="AG21" s="17"/>
       <c r="AH21" s="17"/>
       <c r="AI21" s="15"/>
-      <c r="AJ21" s="35" t="s">
-        <v>16</v>
-      </c>
+      <c r="AJ21" s="35"/>
       <c r="AK21" s="17"/>
       <c r="AL21" s="17"/>
       <c r="AM21" s="17"/>
@@ -1788,22 +1808,20 @@
       <c r="A22" s="2"/>
       <c r="B22" s="3"/>
       <c r="C22" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22" s="17"/>
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
       <c r="G22" s="17"/>
-      <c r="H22" s="16">
-        <v>45</v>
-      </c>
+      <c r="H22" s="16"/>
       <c r="I22" s="17"/>
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
       <c r="L22" s="17"/>
       <c r="M22" s="15"/>
       <c r="N22" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O22" s="17"/>
       <c r="P22" s="17"/>
@@ -1820,9 +1838,9 @@
       <c r="AA22" s="17"/>
       <c r="AB22" s="17"/>
       <c r="AC22" s="15"/>
-      <c r="AD22" s="19">
-        <f>SUM(AD7:AI12,AD17:AI18)/8</f>
-        <v>0</v>
+      <c r="AD22" s="19" t="str">
+        <f>IF(COUNT(AD7:AI12,AD17:AI18)=8,SUM(AD7:AI12,AD17:AI18)/8,"")</f>
+        <v/>
       </c>
       <c r="AE22" s="17"/>
       <c r="AF22" s="17"/>
@@ -1879,7 +1897,7 @@
     </row>
     <row r="24" spans="1:40" ht="12.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -1908,7 +1926,7 @@
     </row>
     <row r="25" spans="1:40" ht="12.75" customHeight="1">
       <c r="A25" s="39" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -1941,7 +1959,7 @@
       </c>
       <c r="W25" s="15"/>
       <c r="Y25" s="20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Z25" s="21"/>
       <c r="AA25" s="21"/>
@@ -1961,7 +1979,7 @@
     </row>
     <row r="26" spans="1:40" ht="12.75" customHeight="1">
       <c r="A26" s="42" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -1986,7 +2004,7 @@
       <c r="V26" s="44"/>
       <c r="W26" s="15"/>
       <c r="Y26" s="45" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z26" s="21"/>
       <c r="AA26" s="21"/>
@@ -2008,7 +2026,7 @@
     </row>
     <row r="27" spans="1:40" ht="12.75" customHeight="1">
       <c r="A27" s="42" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -2033,7 +2051,7 @@
       <c r="V27" s="44"/>
       <c r="W27" s="15"/>
       <c r="Y27" s="45" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="Z27" s="21"/>
       <c r="AA27" s="21"/>
@@ -2055,7 +2073,7 @@
     </row>
     <row r="28" spans="1:40" ht="12.75" customHeight="1">
       <c r="A28" s="42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -2080,7 +2098,7 @@
       <c r="V28" s="44"/>
       <c r="W28" s="15"/>
       <c r="Y28" s="45" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Z28" s="21"/>
       <c r="AA28" s="21"/>
@@ -2102,7 +2120,7 @@
     </row>
     <row r="29" spans="1:40" ht="12.75" customHeight="1">
       <c r="A29" s="42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -2127,7 +2145,7 @@
       <c r="V29" s="44"/>
       <c r="W29" s="15"/>
       <c r="Y29" s="45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="Z29" s="21"/>
       <c r="AA29" s="21"/>
@@ -2149,7 +2167,7 @@
     </row>
     <row r="30" spans="1:40" ht="12.75" customHeight="1">
       <c r="A30" s="42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -2174,7 +2192,7 @@
       <c r="V30" s="44"/>
       <c r="W30" s="15"/>
       <c r="Y30" s="45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="Z30" s="21"/>
       <c r="AA30" s="21"/>
@@ -2196,7 +2214,7 @@
     </row>
     <row r="31" spans="1:40" ht="12.75" customHeight="1">
       <c r="A31" s="42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -2222,7 +2240,7 @@
       <c r="W31" s="15"/>
       <c r="X31" s="10"/>
       <c r="Y31" s="45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Z31" s="21"/>
       <c r="AA31" s="21"/>
@@ -2244,7 +2262,7 @@
     </row>
     <row r="32" spans="1:40" ht="12.75" customHeight="1">
       <c r="A32" s="42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="17"/>
       <c r="C32" s="17"/>
@@ -2272,7 +2290,7 @@
     </row>
     <row r="33" spans="1:40" ht="12.75" customHeight="1">
       <c r="A33" s="42" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B33" s="17"/>
       <c r="C33" s="17"/>
@@ -2300,7 +2318,7 @@
     </row>
     <row r="34" spans="1:40" ht="12.75" customHeight="1">
       <c r="A34" s="42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
@@ -2328,7 +2346,7 @@
     </row>
     <row r="35" spans="1:40" ht="12.75" customHeight="1">
       <c r="A35" s="42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B35" s="17"/>
       <c r="C35" s="17"/>
@@ -2356,7 +2374,7 @@
     </row>
     <row r="36" spans="1:40" ht="12.75" customHeight="1">
       <c r="A36" s="42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B36" s="17"/>
       <c r="C36" s="17"/>
@@ -2384,7 +2402,7 @@
     </row>
     <row r="37" spans="1:40" ht="12.75" customHeight="1">
       <c r="A37" s="42" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B37" s="17"/>
       <c r="C37" s="17"/>
@@ -2410,7 +2428,7 @@
       <c r="W37" s="15"/>
       <c r="X37" s="10"/>
       <c r="AC37" s="46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AD37" s="21"/>
       <c r="AE37" s="21"/>
@@ -2424,8 +2442,8 @@
       <c r="AM37" s="21"/>
     </row>
     <row r="38" spans="1:40" ht="12.75" customHeight="1">
-      <c r="A38" s="50" t="s">
-        <v>55</v>
+      <c r="A38" s="48" t="s">
+        <v>54</v>
       </c>
       <c r="B38" s="17"/>
       <c r="C38" s="17"/>
@@ -2465,7 +2483,7 @@
       <c r="AD38" s="9"/>
       <c r="AE38" s="9"/>
       <c r="AF38" s="47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AG38" s="21"/>
       <c r="AH38" s="21"/>
@@ -2519,55 +2537,55 @@
     </row>
     <row r="40" spans="1:40" ht="12.75" customHeight="1">
       <c r="A40" s="49" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B40" s="21"/>
       <c r="C40" s="21"/>
       <c r="D40" s="21"/>
       <c r="E40" s="21"/>
       <c r="F40" s="21"/>
-      <c r="G40" s="48" t="s">
+      <c r="G40" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="H40" s="29"/>
+      <c r="I40" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="H40" s="29"/>
-      <c r="I40" s="48" t="s">
+      <c r="J40" s="29"/>
+      <c r="K40" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="J40" s="29"/>
-      <c r="K40" s="48" t="s">
+      <c r="L40" s="29"/>
+      <c r="M40" s="50" t="s">
         <v>60</v>
       </c>
-      <c r="L40" s="29"/>
-      <c r="M40" s="48" t="s">
+      <c r="N40" s="29"/>
+      <c r="O40" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="N40" s="29"/>
-      <c r="O40" s="48" t="s">
+      <c r="P40" s="29"/>
+      <c r="Q40" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="48" t="s">
+      <c r="R40" s="29"/>
+      <c r="S40" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="R40" s="29"/>
-      <c r="S40" s="48" t="s">
+      <c r="T40" s="29"/>
+      <c r="U40" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="T40" s="29"/>
-      <c r="U40" s="48" t="s">
+      <c r="V40" s="29"/>
+      <c r="W40" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="V40" s="29"/>
-      <c r="W40" s="48" t="s">
+      <c r="X40" s="29"/>
+      <c r="Y40" s="50" t="s">
         <v>66</v>
       </c>
-      <c r="X40" s="29"/>
-      <c r="Y40" s="48" t="s">
+      <c r="Z40" s="29"/>
+      <c r="AA40" s="50" t="s">
         <v>67</v>
-      </c>
-      <c r="Z40" s="29"/>
-      <c r="AA40" s="48" t="s">
-        <v>68</v>
       </c>
       <c r="AB40" s="29"/>
       <c r="AC40" s="49"/>
@@ -2583,7 +2601,7 @@
     </row>
     <row r="41" spans="1:40" ht="12.75" customHeight="1">
       <c r="A41" s="52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
@@ -2630,11 +2648,11 @@
         <v>16</v>
       </c>
       <c r="Z41" s="15"/>
-      <c r="AA41" s="44">
-        <f t="shared" ref="AA41:AA43" si="1">SUM(G41:Z41)</f>
+      <c r="AA41" s="55">
+        <f>SUM(G41:Z41)</f>
         <v>200</v>
       </c>
-      <c r="AB41" s="15"/>
+      <c r="AB41" s="56"/>
       <c r="AC41" s="53"/>
       <c r="AD41" s="21"/>
       <c r="AG41" s="10"/>
@@ -2648,7 +2666,7 @@
     </row>
     <row r="42" spans="1:40" ht="12.75" customHeight="1">
       <c r="A42" s="52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -2676,7 +2694,7 @@
       <c r="Y42" s="51"/>
       <c r="Z42" s="15"/>
       <c r="AA42" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="AA42:AA43" si="5">SUM(G42:Z42)</f>
         <v>0</v>
       </c>
       <c r="AB42" s="15"/>
@@ -2685,7 +2703,7 @@
     </row>
     <row r="43" spans="1:40" ht="12.75" customHeight="1">
       <c r="A43" s="52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B43" s="17"/>
       <c r="C43" s="17"/>
@@ -2713,7 +2731,7 @@
       <c r="Y43" s="43"/>
       <c r="Z43" s="15"/>
       <c r="AA43" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB43" s="15"/>
@@ -3805,6 +3823,12 @@
     <mergeCell ref="S41:T41"/>
     <mergeCell ref="U41:V41"/>
     <mergeCell ref="W41:X41"/>
+    <mergeCell ref="S40:T40"/>
+    <mergeCell ref="U40:V40"/>
+    <mergeCell ref="W40:X40"/>
+    <mergeCell ref="Y40:Z40"/>
+    <mergeCell ref="AA40:AB40"/>
+    <mergeCell ref="AC40:AD40"/>
     <mergeCell ref="R32:S32"/>
     <mergeCell ref="T32:U32"/>
     <mergeCell ref="V32:W32"/>
@@ -3819,6 +3843,10 @@
     <mergeCell ref="T34:U34"/>
     <mergeCell ref="V34:W34"/>
     <mergeCell ref="A35:O35"/>
+    <mergeCell ref="R33:S33"/>
+    <mergeCell ref="T33:U33"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="R35:S35"/>
     <mergeCell ref="Q43:R43"/>
     <mergeCell ref="S43:T43"/>
     <mergeCell ref="U43:V43"/>
@@ -3852,12 +3880,6 @@
     <mergeCell ref="I41:J41"/>
     <mergeCell ref="G42:H42"/>
     <mergeCell ref="I42:J42"/>
-    <mergeCell ref="S40:T40"/>
-    <mergeCell ref="U40:V40"/>
-    <mergeCell ref="W40:X40"/>
-    <mergeCell ref="Y40:Z40"/>
-    <mergeCell ref="AA40:AB40"/>
-    <mergeCell ref="AC40:AD40"/>
     <mergeCell ref="A37:O37"/>
     <mergeCell ref="A38:O38"/>
     <mergeCell ref="P38:Q38"/>
@@ -3869,10 +3891,6 @@
     <mergeCell ref="M40:N40"/>
     <mergeCell ref="R37:S37"/>
     <mergeCell ref="T37:U37"/>
-    <mergeCell ref="R33:S33"/>
-    <mergeCell ref="T33:U33"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="R35:S35"/>
     <mergeCell ref="AC37:AM37"/>
     <mergeCell ref="AF38:AK38"/>
     <mergeCell ref="R27:S27"/>
@@ -3971,7 +3989,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.9" bottom="0.25" header="0" footer="0"/>
-  <pageSetup scale="97" orientation="portrait"/>
+  <pageSetup scale="97" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L       &amp;C BACOLOD TRINITY CHRISTIAN SCHOOL, INC. Villa Angela Subdivision, Phase 3, Bacolod City DepEd Recognition No. 001 s. 1981, 006 s. 1983 ACCREDITED BY ACSCU-ACI, CERTIFIED BY FAAP&amp;RDepEd Form 138</oddHeader>
   </headerFooter>

</xml_diff>